<commit_message>
chore: daily SAM report 2026-10-26
</commit_message>
<xml_diff>
--- a/docs/v/SAM-daily-latest.xlsx
+++ b/docs/v/SAM-daily-latest.xlsx
@@ -8,14 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Daily Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Day 2026-10-25" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Day 2026-10-26" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="All Notices" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="First Seen By Day" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Run Log" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$E$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Day 2026-10-25'!$A$1:$R$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Day 2026-10-26'!$A$1:$R$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Notices'!$A$1:$R$130</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'First Seen By Day'!$A$1:$R$130</definedName>
   </definedNames>
@@ -513,7 +513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -534,7 +534,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -544,99 +544,99 @@
         <v>39</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>45</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -646,14 +646,14 @@
         <v>45</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -663,31 +663,31 @@
         <v>45</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -697,38 +697,38 @@
         <v>46</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>4</v>
@@ -738,24 +738,24 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
@@ -899,7 +899,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr"/>
@@ -964,14 +964,14 @@
       </c>
       <c r="R2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr"/>
@@ -1036,14 +1036,14 @@
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr"/>
@@ -1108,14 +1108,14 @@
       </c>
       <c r="R4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
@@ -1180,14 +1180,14 @@
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
@@ -1252,14 +1252,14 @@
       </c>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
@@ -1324,14 +1324,14 @@
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
@@ -1396,14 +1396,14 @@
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
@@ -1468,14 +1468,14 @@
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr"/>
@@ -1536,14 +1536,14 @@
       </c>
       <c r="R10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr"/>
@@ -1608,14 +1608,14 @@
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr"/>
@@ -1680,14 +1680,14 @@
       </c>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr"/>
@@ -1748,14 +1748,14 @@
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr"/>
@@ -1820,14 +1820,14 @@
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr"/>
@@ -1892,14 +1892,14 @@
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr"/>
@@ -1964,14 +1964,14 @@
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr"/>
@@ -2036,14 +2036,14 @@
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr"/>
@@ -2108,14 +2108,14 @@
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr"/>
@@ -2180,14 +2180,14 @@
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr"/>
@@ -2252,14 +2252,14 @@
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr"/>
@@ -2324,14 +2324,14 @@
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr"/>
@@ -2396,14 +2396,14 @@
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr"/>
@@ -2468,14 +2468,14 @@
       </c>
       <c r="R23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr"/>
@@ -2540,14 +2540,14 @@
       </c>
       <c r="R24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr"/>
@@ -2612,14 +2612,14 @@
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr"/>
@@ -2684,14 +2684,14 @@
       </c>
       <c r="R26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr"/>
@@ -2756,14 +2756,14 @@
       </c>
       <c r="R27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr"/>
@@ -2828,14 +2828,14 @@
       </c>
       <c r="R28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr"/>
@@ -2900,14 +2900,14 @@
       </c>
       <c r="R29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr"/>
@@ -2972,14 +2972,14 @@
       </c>
       <c r="R30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr"/>
@@ -3044,14 +3044,14 @@
       </c>
       <c r="R31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr"/>
@@ -3116,14 +3116,14 @@
       </c>
       <c r="R32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
@@ -3188,14 +3188,14 @@
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr"/>
@@ -3260,14 +3260,14 @@
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
@@ -3332,14 +3332,14 @@
       </c>
       <c r="R35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr"/>
@@ -3404,14 +3404,14 @@
       </c>
       <c r="R36" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr"/>
@@ -3476,14 +3476,14 @@
       </c>
       <c r="R37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr"/>
@@ -3548,14 +3548,14 @@
       </c>
       <c r="R38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
@@ -3620,14 +3620,14 @@
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr"/>
@@ -3692,7 +3692,7 @@
       </c>
       <c r="R40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3867,7 +3867,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr"/>
@@ -3932,14 +3932,14 @@
       </c>
       <c r="R2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr"/>
@@ -4004,14 +4004,14 @@
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr"/>
@@ -4076,14 +4076,14 @@
       </c>
       <c r="R4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
@@ -4148,14 +4148,14 @@
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
@@ -4220,14 +4220,14 @@
       </c>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
@@ -4292,14 +4292,14 @@
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
@@ -4364,14 +4364,14 @@
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
@@ -4436,14 +4436,14 @@
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr"/>
@@ -4508,14 +4508,14 @@
       </c>
       <c r="R10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr"/>
@@ -4576,14 +4576,14 @@
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr"/>
@@ -4648,14 +4648,14 @@
       </c>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr"/>
@@ -4720,14 +4720,14 @@
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr"/>
@@ -4788,14 +4788,14 @@
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr"/>
@@ -4860,14 +4860,14 @@
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr"/>
@@ -4932,14 +4932,14 @@
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr"/>
@@ -5004,14 +5004,14 @@
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr"/>
@@ -5076,14 +5076,14 @@
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr"/>
@@ -5148,14 +5148,14 @@
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr"/>
@@ -5220,14 +5220,14 @@
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr"/>
@@ -5292,14 +5292,14 @@
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr"/>
@@ -5364,14 +5364,14 @@
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr"/>
@@ -5436,14 +5436,14 @@
       </c>
       <c r="R23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr"/>
@@ -5508,14 +5508,14 @@
       </c>
       <c r="R24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr"/>
@@ -5580,14 +5580,14 @@
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr"/>
@@ -5652,14 +5652,14 @@
       </c>
       <c r="R26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr"/>
@@ -5724,14 +5724,14 @@
       </c>
       <c r="R27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr"/>
@@ -5796,14 +5796,14 @@
       </c>
       <c r="R28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr"/>
@@ -5868,14 +5868,14 @@
       </c>
       <c r="R29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr"/>
@@ -5940,14 +5940,14 @@
       </c>
       <c r="R30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr"/>
@@ -6012,14 +6012,14 @@
       </c>
       <c r="R31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr"/>
@@ -6084,14 +6084,14 @@
       </c>
       <c r="R32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
@@ -6156,14 +6156,14 @@
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr"/>
@@ -6228,14 +6228,14 @@
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
@@ -6300,14 +6300,14 @@
       </c>
       <c r="R35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr"/>
@@ -6372,14 +6372,14 @@
       </c>
       <c r="R36" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr"/>
@@ -6444,14 +6444,14 @@
       </c>
       <c r="R37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr"/>
@@ -6516,14 +6516,14 @@
       </c>
       <c r="R38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
@@ -6588,14 +6588,14 @@
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr"/>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="R40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -13426,7 +13426,7 @@
       </c>
       <c r="R2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -13498,7 +13498,7 @@
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -13570,7 +13570,7 @@
       </c>
       <c r="R4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -13642,7 +13642,7 @@
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -13714,7 +13714,7 @@
       </c>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -13786,7 +13786,7 @@
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -13858,7 +13858,7 @@
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -13930,7 +13930,7 @@
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14070,7 +14070,7 @@
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14142,7 +14142,7 @@
       </c>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14214,7 +14214,7 @@
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14282,7 +14282,7 @@
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14354,7 +14354,7 @@
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14426,7 +14426,7 @@
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14498,7 +14498,7 @@
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14642,7 +14642,7 @@
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14714,7 +14714,7 @@
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14786,7 +14786,7 @@
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14858,7 +14858,7 @@
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -14930,7 +14930,7 @@
       </c>
       <c r="R23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15002,7 +15002,7 @@
       </c>
       <c r="R24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15074,7 +15074,7 @@
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15146,7 +15146,7 @@
       </c>
       <c r="R26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15218,7 +15218,7 @@
       </c>
       <c r="R27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15290,7 +15290,7 @@
       </c>
       <c r="R28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15434,7 +15434,7 @@
       </c>
       <c r="R30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15650,7 +15650,7 @@
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15722,7 +15722,7 @@
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -15938,7 +15938,7 @@
       </c>
       <c r="R37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -16010,7 +16010,7 @@
       </c>
       <c r="R38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -16082,7 +16082,7 @@
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -16154,7 +16154,7 @@
       </c>
       <c r="R40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -16226,7 +16226,7 @@
       </c>
       <c r="R41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -16370,7 +16370,7 @@
       </c>
       <c r="R43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -16586,7 +16586,7 @@
       </c>
       <c r="R46" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -16946,7 +16946,7 @@
       </c>
       <c r="R51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -17662,7 +17662,7 @@
       </c>
       <c r="R61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -18238,7 +18238,7 @@
       </c>
       <c r="R69" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -18310,7 +18310,7 @@
       </c>
       <c r="R70" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -22807,22 +22807,22 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25_092210</t>
+          <t>2026-10-26_093449</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -22845,22 +22845,22 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24_092128</t>
+          <t>2026-10-25_092210</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -22870,7 +22870,7 @@
         <v>39</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>3</v>
@@ -22883,32 +22883,32 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23_092806</t>
+          <t>2026-10-24_092128</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>29</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>3</v>
@@ -22921,32 +22921,32 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22_092931</t>
+          <t>2026-10-23_092806</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>29</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>3</v>
@@ -22959,32 +22959,32 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21_092743</t>
+          <t>2026-10-22_092931</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>29</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>3</v>
@@ -22997,7 +22997,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-21_012830</t>
+          <t>2026-10-21_092743</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -23022,7 +23022,7 @@
         <v>42</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>3</v>
@@ -23035,32 +23035,32 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20_162138</t>
+          <t>2026-10-21_012830</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>29</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>3</v>
@@ -23073,7 +23073,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20_141035</t>
+          <t>2026-10-20_162138</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -23092,13 +23092,13 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>3</v>
@@ -23111,32 +23111,32 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19_161731</t>
+          <t>2026-10-20_141035</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>24</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>3</v>
@@ -23149,22 +23149,22 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18_130358</t>
+          <t>2026-10-19_161731</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -23174,7 +23174,7 @@
         <v>45</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>3</v>
@@ -23187,22 +23187,22 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17_124531</t>
+          <t>2026-10-18_130358</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -23212,7 +23212,7 @@
         <v>45</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>3</v>
@@ -23225,32 +23225,32 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-16_134806</t>
+          <t>2026-10-17_124531</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
         <v>24</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>3</v>
@@ -23263,22 +23263,22 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15_140128</t>
+          <t>2026-10-16_134806</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
@@ -23288,7 +23288,7 @@
         <v>46</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>3</v>
@@ -23301,32 +23301,32 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_142359</t>
+          <t>2026-10-15_140128</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>24</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H15" s="3" t="n">
         <v>3</v>
@@ -23339,29 +23339,29 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13_164653</t>
+          <t>2026-10-14_142359</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
         <v>24</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>4</v>
@@ -23377,32 +23377,32 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12_184410</t>
+          <t>2026-10-13_164653</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>24</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>3</v>
@@ -23415,22 +23415,22 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-11_152459</t>
+          <t>2026-10-12_184410</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">

</xml_diff>